<commit_message>
feat(migracion): soporte de estados asignado/pendiente_asignar/sin_rcl en identidad_legacy
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/identidad_legacy_test.xlsx
+++ b/tests/fixtures/identidad_legacy_test.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -569,79 +569,95 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>MZ11-C001</v>
+      </c>
+      <c r="B22" t="str">
         <v/>
-      </c>
-      <c r="B22" t="str">
-        <v>RCL300-C001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MZ11-C001</v>
+        <v>MZ11-C003</v>
       </c>
       <c r="B23" t="str">
-        <v/>
+        <v>*</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MZ1-C1</v>
+        <v>MZ11-C004</v>
       </c>
       <c r="B24" t="str">
-        <v>RCL301-C001</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MZ11-C002</v>
+        <v/>
       </c>
       <c r="B25" t="str">
-        <v>XYZ301-C001</v>
+        <v>RCL300-C001</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MZ12-C001</v>
+        <v>MZ1-C1</v>
       </c>
       <c r="B26" t="str">
-        <v>RCL302-C001</v>
+        <v>RCL301-C001</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MZ12-C001</v>
+        <v>MZ11-C002</v>
       </c>
       <c r="B27" t="str">
-        <v>RCL303-C001</v>
+        <v>XYZ301-C001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MZ12-C002</v>
+        <v>MZ12-C001</v>
       </c>
       <c r="B28" t="str">
-        <v>RCL304-C001</v>
+        <v>RCL302-C001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MZ12-C003</v>
+        <v>MZ12-C001</v>
       </c>
       <c r="B29" t="str">
-        <v>RCL304-C001</v>
+        <v>RCL303-C001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
+        <v>MZ12-C002</v>
+      </c>
+      <c r="B30" t="str">
+        <v>RCL304-C001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>MZ12-C003</v>
+      </c>
+      <c r="B31" t="str">
+        <v>RCL304-C001</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
         <v>MZ12-C005</v>
       </c>
-      <c r="B30" t="str">
+      <c r="B32" t="str">
         <v>RCL999-C999</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(migracion): identidad_legacy a nivel de sub-posicion (nivel/subnivel)
El archivo real del cliente trae la identidad RCL<->MZ a nivel de
sub-posicion (MZ01-C001-N01-1 <-> RCL112-C001-N01-1, 5 sub-niveles por
columna), no por columna como asumia F1. PK, unique parcial de RCL y el
CHECK de coherencia se extienden a (pasillo, columna, nivel, subnivel).
La deteccion de duplicados ahora compara la sub-posicion completa: el
mismo pasillo+columna en un nivel distinto ya no se marca como error.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/identidad_legacy_test.xlsx
+++ b/tests/fixtures/identidad_legacy_test.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,255 +409,135 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>MZ01-C001</v>
+        <v>MZ01-C001-N01-1</v>
       </c>
       <c r="B2" t="str">
-        <v>RCL121-C001</v>
+        <v>RCL112-C001-N01-1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MZ01-C002</v>
+        <v>MZ01-C001-N02-1</v>
       </c>
       <c r="B3" t="str">
-        <v>RCL122-C001</v>
+        <v>RCL112-C001-N02-1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MZ01-C003</v>
+        <v>MZ01-C002-N01-1</v>
       </c>
       <c r="B4" t="str">
-        <v>RCL122-C002</v>
+        <v>RCL113-C001-N01-1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MZ02-C001</v>
+        <v>MZ02-C018-N01-1</v>
       </c>
       <c r="B5" t="str">
-        <v>RCL130-001</v>
+        <v>RCL146-C002-N01-1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MZ02-C002</v>
+        <v>mz09-C001-n01-1</v>
       </c>
       <c r="B6" t="str">
-        <v>RCL130-002</v>
+        <v>n/a-n01-1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MZ02-C010</v>
+        <v>MZ09-C002-N01-1</v>
       </c>
       <c r="B7" t="str">
-        <v>RCL140-C001</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MZ03-C001</v>
+        <v>MZ10-C001-N01-1</v>
       </c>
       <c r="B8" t="str">
-        <v>RCL150-C001</v>
+        <v>*</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MZ03-C015</v>
+        <v>MZ10-C002-N01-1</v>
       </c>
       <c r="B9" t="str">
-        <v>RCL151-C003</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MZ04-C001</v>
+        <v>MZ1-C001-N01-1</v>
       </c>
       <c r="B10" t="str">
-        <v>RCL160-001</v>
+        <v>RCL999-C001-N01-1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MZ04-C020</v>
+        <v>MZ11-C001-N01-1</v>
       </c>
       <c r="B11" t="str">
-        <v>RCL161-C002</v>
+        <v>RCLABC-C001-N01-1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MZ05-C001</v>
+        <v/>
       </c>
       <c r="B12" t="str">
-        <v>RCL170-C001</v>
+        <v>RCL120-C001-N01-1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MZ05-C011</v>
+        <v>MZ12-C001-N01-1</v>
       </c>
       <c r="B13" t="str">
-        <v>RCL171-002</v>
+        <v>RCL150-C001-N01-1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MZ06-C001</v>
+        <v>MZ12-C001-N01-1</v>
       </c>
       <c r="B14" t="str">
-        <v>RCL180-C001</v>
+        <v>RCL151-C001-N01-1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MZ06-C030</v>
+        <v>MZ12-C002-N01-1</v>
       </c>
       <c r="B15" t="str">
-        <v>RCL181-C001</v>
+        <v>RCL160-C001-N01-1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MZ07-C001</v>
+        <v>MZ12-C003-N01-1</v>
       </c>
       <c r="B16" t="str">
-        <v>RCL190-001</v>
+        <v>RCL160-C001-N01-1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MZ07-C025</v>
+        <v>MZ12-C005-N01-1</v>
       </c>
       <c r="B17" t="str">
-        <v>RCL191-C002</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>MZ08-C001</v>
-      </c>
-      <c r="B18" t="str">
-        <v>RCL200-C001</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>MZ08-C041</v>
-      </c>
-      <c r="B19" t="str">
-        <v>RCL208-C002</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>MZ09-C001</v>
-      </c>
-      <c r="B20" t="str">
-        <v>RCL210-001</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v xml:space="preserve">  MZ10-C001  </v>
-      </c>
-      <c r="B21" t="str">
-        <v xml:space="preserve">  RCL220-C001  </v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>MZ11-C001</v>
-      </c>
-      <c r="B22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>MZ11-C003</v>
-      </c>
-      <c r="B23" t="str">
-        <v>*</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>MZ11-C004</v>
-      </c>
-      <c r="B24" t="str">
-        <v>N/A</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v/>
-      </c>
-      <c r="B25" t="str">
-        <v>RCL300-C001</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>MZ1-C1</v>
-      </c>
-      <c r="B26" t="str">
-        <v>RCL301-C001</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>MZ11-C002</v>
-      </c>
-      <c r="B27" t="str">
-        <v>XYZ301-C001</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>MZ12-C001</v>
-      </c>
-      <c r="B28" t="str">
-        <v>RCL302-C001</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>MZ12-C001</v>
-      </c>
-      <c r="B29" t="str">
-        <v>RCL303-C001</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>MZ12-C002</v>
-      </c>
-      <c r="B30" t="str">
-        <v>RCL304-C001</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>MZ12-C003</v>
-      </c>
-      <c r="B31" t="str">
-        <v>RCL304-C001</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>MZ12-C005</v>
-      </c>
-      <c r="B32" t="str">
-        <v>RCL999-C999</v>
+        <v>RCL999-C999-N01-1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>